<commit_message>
Regenerate results after 0002-lp-bottleneck-stage2-face (Windows run)
</commit_message>
<xml_diff>
--- a/results/tables/excel/table_A3_robustness_suite.xlsx
+++ b/results/tables/excel/table_A3_robustness_suite.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X12"/>
+  <dimension ref="A1:AC12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -521,30 +521,55 @@
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
+          <t>bottleneck_tight</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>bottleneck_sufficient</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>bottleneck_necessary</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
           <t>bottleneck_identified</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>with_bottleneck</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>stage2_optimum_unique</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>stage3_active</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>stage3_inactive_face_not_point</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>stage3_active_share</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>median_relative_reduction_when_active</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>median_ratios_moved_when_active</t>
         </is>
@@ -618,15 +643,30 @@
         <v>40</v>
       </c>
       <c r="U2" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="V2" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="W2" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="X2" t="n">
+        <v>40</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -698,15 +738,30 @@
         <v>25</v>
       </c>
       <c r="U3" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="V3" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="W3" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="X3" t="n">
+        <v>25</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -778,15 +833,30 @@
         <v>25</v>
       </c>
       <c r="U4" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="V4" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="W4" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="X4" t="n">
+        <v>25</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -858,15 +928,30 @@
         <v>30</v>
       </c>
       <c r="U5" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="V5" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="W5" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="X5" t="n">
+        <v>30</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -938,15 +1023,30 @@
         <v>20</v>
       </c>
       <c r="U6" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="V6" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="W6" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="X6" t="n">
+        <v>20</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1018,15 +1118,30 @@
         <v>30</v>
       </c>
       <c r="U7" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="V7" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="W7" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="X7" t="n">
+        <v>30</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1098,15 +1213,30 @@
         <v>30</v>
       </c>
       <c r="U8" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="V8" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="W8" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="X8" t="n">
+        <v>30</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1178,15 +1308,30 @@
         <v>80</v>
       </c>
       <c r="U9" t="n">
+        <v>80</v>
+      </c>
+      <c r="V9" t="n">
+        <v>80</v>
+      </c>
+      <c r="W9" t="n">
+        <v>80</v>
+      </c>
+      <c r="X9" t="n">
+        <v>24</v>
+      </c>
+      <c r="Y9" t="n">
         <v>38</v>
       </c>
-      <c r="V9" t="n">
+      <c r="Z9" t="n">
+        <v>18</v>
+      </c>
+      <c r="AA9" t="n">
         <v>0.475</v>
       </c>
-      <c r="W9" t="n">
+      <c r="AB9" t="n">
         <v>0.07720062479155906</v>
       </c>
-      <c r="X9" t="n">
+      <c r="AC9" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1258,15 +1403,30 @@
         <v>60</v>
       </c>
       <c r="U10" t="n">
+        <v>60</v>
+      </c>
+      <c r="V10" t="n">
+        <v>60</v>
+      </c>
+      <c r="W10" t="n">
+        <v>60</v>
+      </c>
+      <c r="X10" t="n">
         <v>21</v>
       </c>
-      <c r="V10" t="n">
+      <c r="Y10" t="n">
+        <v>21</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>18</v>
+      </c>
+      <c r="AA10" t="n">
         <v>0.35</v>
       </c>
-      <c r="W10" t="n">
+      <c r="AB10" t="n">
         <v>0.07887763662780092</v>
       </c>
-      <c r="X10" t="n">
+      <c r="AC10" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1338,15 +1498,30 @@
         <v>60</v>
       </c>
       <c r="U11" t="n">
+        <v>60</v>
+      </c>
+      <c r="V11" t="n">
+        <v>60</v>
+      </c>
+      <c r="W11" t="n">
+        <v>60</v>
+      </c>
+      <c r="X11" t="n">
+        <v>58</v>
+      </c>
+      <c r="Y11" t="n">
         <v>2</v>
       </c>
-      <c r="V11" t="n">
+      <c r="Z11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA11" t="n">
         <v>0.03333333333333333</v>
       </c>
-      <c r="W11" t="n">
+      <c r="AB11" t="n">
         <v>0.02271534936768814</v>
       </c>
-      <c r="X11" t="n">
+      <c r="AC11" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1418,15 +1593,30 @@
         <v>400</v>
       </c>
       <c r="U12" t="n">
+        <v>400</v>
+      </c>
+      <c r="V12" t="n">
+        <v>400</v>
+      </c>
+      <c r="W12" t="n">
+        <v>400</v>
+      </c>
+      <c r="X12" t="n">
+        <v>303</v>
+      </c>
+      <c r="Y12" t="n">
         <v>61</v>
       </c>
-      <c r="V12" t="n">
+      <c r="Z12" t="n">
+        <v>36</v>
+      </c>
+      <c r="AA12" t="n">
         <v>0.1525</v>
       </c>
-      <c r="W12" t="n">
+      <c r="AB12" t="n">
         <v>0.07418209978586164</v>
       </c>
-      <c r="X12" t="n">
+      <c r="AC12" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>